<commit_message>
feat: update accurate and active official websites for all 23 schools
</commit_message>
<xml_diff>
--- a/Tong_hop_truong_GDNN_tinh_Ninh_Binh_moi_2026.xlsx
+++ b/Tong_hop_truong_GDNN_tinh_Ninh_Binh_moi_2026.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="390">
   <si>
     <t>TỔNG HỢP DANH SÁCH 23 CƠ SỞ GIÁO DỤC NGHỀ NGHIỆP TỈNH NINH BÌNH (28 CỘT CHUẨN ADMIN)</t>
   </si>
@@ -124,7 +124,7 @@
     <t>0912 137 176</t>
   </si>
   <si>
-    <t>https://cdktcnnb.edu.vn</t>
+    <t>https://ncet.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: Đinh Văn Hoản</t>
@@ -148,7 +148,7 @@
     <t>0229 387 1042</t>
   </si>
   <si>
-    <t>https://cdyteninhbinh.edu.vn</t>
+    <t>https://cdyteninhbinh.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: TS. Nguyễn Thị Thu Hà</t>
@@ -172,7 +172,7 @@
     <t>0228 384 9234</t>
   </si>
   <si>
-    <t>http://vhntnamdinh.edu.vn</t>
+    <t>http://cdvhntdlnd.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: ThS. Trần Thị Kim Oanh</t>
@@ -196,7 +196,7 @@
     <t>0917 620 019</t>
   </si>
   <si>
-    <t>http://caodanglilama1.edu.vn</t>
+    <t>https://caodanglilama1.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: Phạm Duy Bảy</t>
@@ -220,7 +220,7 @@
     <t>0229 377 0795</t>
   </si>
   <si>
-    <t>http://cdcodiennn.edu.vn</t>
+    <t>https://caee.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: Dương Văn Cường</t>
@@ -244,7 +244,7 @@
     <t>0983 703 936</t>
   </si>
   <si>
-    <t>http://cdcnnd.edu.vn</t>
+    <t>http://www.cnd.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: Thầy Nguyễn Duy Phấn</t>
@@ -265,7 +265,7 @@
     <t>0912 180 984</t>
   </si>
   <si>
-    <t>http://cdxdnd.edu.vn</t>
+    <t>http://cdxdnd.edu.vn/</t>
   </si>
   <si>
     <t>Phó Hiệu trưởng phụ trách: Lương Văn Doanh</t>
@@ -289,7 +289,7 @@
     <t>0226 385 4123</t>
   </si>
   <si>
-    <t>http://lamnghieptw.edu.vn</t>
+    <t>https://cdcongnghekinhte.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: ThS. Nguyễn Văn Thành</t>
@@ -313,7 +313,7 @@
     <t>0226 385 2772</t>
   </si>
   <si>
-    <t>https://vov.edu.vn</t>
+    <t>https://vov.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: TS. Nguyễn Văn Sơn</t>
@@ -337,7 +337,7 @@
     <t>0226 385 2769</t>
   </si>
   <si>
-    <t>http://thuyloibb.edu.vn</t>
+    <t>https://mwc.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: ThS. Phạm Gia Điệp</t>
@@ -358,7 +358,7 @@
     <t>0228 383 4465</t>
   </si>
   <si>
-    <t>http://caodang20.edu.vn</t>
+    <t>https://caodang20.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: Trần Quang Dũng</t>
@@ -382,7 +382,7 @@
     <t>0226 730 0999</t>
   </si>
   <si>
-    <t>https://caodang.fpt.edu.vn</t>
+    <t>https://caodang.fpt.edu.vn/</t>
   </si>
   <si>
     <t>Giám đốc: Vũ Chí Thành</t>
@@ -403,9 +403,6 @@
     <t>0228 384 8562</t>
   </si>
   <si>
-    <t>http://cddetmaynamdinh.edu.vn</t>
-  </si>
-  <si>
     <t>Hiệu trưởng: ThS. Lê Thị Mai</t>
   </si>
   <si>
@@ -424,7 +421,7 @@
     <t>0228 384 9452</t>
   </si>
   <si>
-    <t>http://cdspnamdinh.edu.vn</t>
+    <t>https://cdspnd.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: TS. Trần Duy Hưng</t>
@@ -448,7 +445,7 @@
     <t>0985 453 868</t>
   </si>
   <si>
-    <t>http://sgtvt.ninhbinh.gov.vn</t>
+    <t>https://www.facebook.com/TTSHLXNB/</t>
   </si>
   <si>
     <t>Hiệu trưởng: Phạm Quang Thể</t>
@@ -472,7 +469,7 @@
     <t>0913 517 988</t>
   </si>
   <si>
-    <t>http://congngheso8.edu.vn</t>
+    <t>https://www.truongtccn8nd.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: Nguyễn Chí Thuấn</t>
@@ -496,7 +493,7 @@
     <t>0988 119 197</t>
   </si>
   <si>
-    <t>http://tccdnb.edu.vn</t>
+    <t>http://tccdnb.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: Dương Mạnh Hiền</t>
@@ -520,7 +517,7 @@
     <t>0918 843 843</t>
   </si>
   <si>
-    <t>http://trungcapdailam.edu.vn</t>
+    <t>https://truongtrungcapdailam.edu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: Trần Thọ Hiền</t>
@@ -541,7 +538,7 @@
     <t>0228 368 6868</t>
   </si>
   <si>
-    <t>https://yduoctonthattung.edu.vn</t>
+    <t>https://truongyduoctonthattung.com.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: BS. Tôn Thất Hưng</t>
@@ -565,7 +562,7 @@
     <t>0913 583 517</t>
   </si>
   <si>
-    <t>http://trungcapquocte.edu.vn</t>
+    <t>https://ivsedu.vn/</t>
   </si>
   <si>
     <t>Hiệu trưởng: Trần Minh Chất</t>
@@ -586,7 +583,7 @@
     <t>0229 386 8899</t>
   </si>
   <si>
-    <t>http://vietucninhbinh.edu.vn</t>
+    <t>https://www.facebook.com/vietuchanam/</t>
   </si>
   <si>
     <t>Hiệu trưởng: ThS. Nguyễn Văn Úc</t>
@@ -610,7 +607,7 @@
     <t>0226 388 3456</t>
   </si>
   <si>
-    <t>http://yduochanam.edu.vn</t>
+    <t>https://yduochanam.blogspot.com/</t>
   </si>
   <si>
     <t>Hiệu trưởng: DS. Trần Thị Minh</t>
@@ -634,9 +631,6 @@
     <t>0229 383 6789</t>
   </si>
   <si>
-    <t>http://kythuatcaonb.edu.vn</t>
-  </si>
-  <si>
     <t>Hiệu trưởng: ThS. Đỗ Văn Cương</t>
   </si>
   <si>
@@ -835,22 +829,22 @@
     <t>Đại học</t>
   </si>
   <si>
+    <t>Phường Châu Sơn</t>
+  </si>
+  <si>
+    <t>Phường Duy Hà</t>
+  </si>
+  <si>
+    <t>Phường Duy Tân</t>
+  </si>
+  <si>
     <t>GDTX</t>
   </si>
   <si>
+    <t>Phường Duy Tiên</t>
+  </si>
+  <si>
     <t>GDTX - GDNN</t>
-  </si>
-  <si>
-    <t>Phường Châu Sơn</t>
-  </si>
-  <si>
-    <t>Phường Duy Hà</t>
-  </si>
-  <si>
-    <t>Phường Duy Tân</t>
-  </si>
-  <si>
-    <t>Phường Duy Tiên</t>
   </si>
   <si>
     <t>Phường Đông A</t>
@@ -2831,7 +2825,7 @@
         <v>127</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="I16" s="9">
         <v>48000.0</v>
@@ -2843,7 +2837,7 @@
         <v>12</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M16" s="9">
         <v>500</v>
@@ -2858,7 +2852,7 @@
         <v>94.0</v>
       </c>
       <c r="Q16" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="R16" s="9">
         <v>68</v>
@@ -2891,12 +2885,12 @@
         <v>0</v>
       </c>
       <c r="AB16" s="7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:28" customHeight="1" ht="26">
       <c r="A17" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B17" s="8" t="s">
         <v>31</v>
@@ -2905,7 +2899,7 @@
         <v>48</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E17" s="8">
         <v>20.4312</v>
@@ -2914,10 +2908,10 @@
         <v>106.1824</v>
       </c>
       <c r="G17" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="H17" s="7" t="s">
         <v>134</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>135</v>
       </c>
       <c r="I17" s="9">
         <v>50000.0</v>
@@ -2929,7 +2923,7 @@
         <v>6</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="M17" s="9">
         <v>550</v>
@@ -2944,7 +2938,7 @@
         <v>92.0</v>
       </c>
       <c r="Q17" s="7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="R17" s="9">
         <v>82</v>
@@ -2977,21 +2971,21 @@
         <v>0</v>
       </c>
       <c r="AB17" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" spans="1:28" customHeight="1" ht="26">
       <c r="A18" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>139</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>140</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>72</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E18" s="8">
         <v>20.409575</v>
@@ -3000,10 +2994,10 @@
         <v>106.14908200000001</v>
       </c>
       <c r="G18" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="H18" s="7" t="s">
         <v>142</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>143</v>
       </c>
       <c r="I18" s="9">
         <v>32000.0</v>
@@ -3015,7 +3009,7 @@
         <v>6</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="M18" s="9">
         <v>400</v>
@@ -3030,7 +3024,7 @@
         <v>93.0</v>
       </c>
       <c r="Q18" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="R18" s="9">
         <v>45</v>
@@ -3063,21 +3057,21 @@
         <v>0</v>
       </c>
       <c r="AB18" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="19" spans="1:28" customHeight="1" ht="26">
       <c r="A19" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="B19" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="7" t="s">
         <v>148</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>149</v>
       </c>
       <c r="E19" s="8">
         <v>20.396133</v>
@@ -3086,10 +3080,10 @@
         <v>106.213331</v>
       </c>
       <c r="G19" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="H19" s="7" t="s">
         <v>150</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>151</v>
       </c>
       <c r="I19" s="9">
         <v>28000.0</v>
@@ -3101,7 +3095,7 @@
         <v>5</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="M19" s="9">
         <v>350</v>
@@ -3116,7 +3110,7 @@
         <v>91.5</v>
       </c>
       <c r="Q19" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="R19" s="9">
         <v>38</v>
@@ -3149,21 +3143,21 @@
         <v>0</v>
       </c>
       <c r="AB19" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="20" spans="1:28" customHeight="1" ht="26">
       <c r="A20" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C20" s="7" t="s">
+      <c r="D20" s="7" t="s">
         <v>156</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>157</v>
       </c>
       <c r="E20" s="8">
         <v>20.249714</v>
@@ -3172,10 +3166,10 @@
         <v>105.995138</v>
       </c>
       <c r="G20" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="H20" s="7" t="s">
         <v>158</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>159</v>
       </c>
       <c r="I20" s="9">
         <v>30000.0</v>
@@ -3187,7 +3181,7 @@
         <v>7</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="M20" s="9">
         <v>420</v>
@@ -3202,7 +3196,7 @@
         <v>94.5</v>
       </c>
       <c r="Q20" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="R20" s="9">
         <v>48</v>
@@ -3235,21 +3229,21 @@
         <v>0</v>
       </c>
       <c r="AB20" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21" spans="1:28" customHeight="1" ht="26">
       <c r="A21" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C21" s="7" t="s">
+      <c r="D21" s="7" t="s">
         <v>164</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>165</v>
       </c>
       <c r="E21" s="8">
         <v>20.458024</v>
@@ -3258,10 +3252,10 @@
         <v>106.187597</v>
       </c>
       <c r="G21" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="H21" s="7" t="s">
         <v>166</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>167</v>
       </c>
       <c r="I21" s="9">
         <v>22000.0</v>
@@ -3273,7 +3267,7 @@
         <v>4</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="M21" s="9">
         <v>280</v>
@@ -3288,7 +3282,7 @@
         <v>90.0</v>
       </c>
       <c r="Q21" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="R21" s="9">
         <v>32</v>
@@ -3321,21 +3315,21 @@
         <v>0</v>
       </c>
       <c r="AB21" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="22" spans="1:28" customHeight="1" ht="26">
       <c r="A22" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>48</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E22" s="8">
         <v>20.4421</v>
@@ -3344,10 +3338,10 @@
         <v>106.1765</v>
       </c>
       <c r="G22" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="H22" s="7" t="s">
         <v>173</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>174</v>
       </c>
       <c r="I22" s="9">
         <v>26000.0</v>
@@ -3359,7 +3353,7 @@
         <v>6</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="M22" s="9">
         <v>380</v>
@@ -3374,7 +3368,7 @@
         <v>93.5</v>
       </c>
       <c r="Q22" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="R22" s="9">
         <v>42</v>
@@ -3407,21 +3401,21 @@
         <v>0</v>
       </c>
       <c r="AB22" s="7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="23" spans="1:28" customHeight="1" ht="26">
       <c r="A23" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C23" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C23" s="7" t="s">
+      <c r="D23" s="7" t="s">
         <v>179</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>180</v>
       </c>
       <c r="E23" s="8">
         <v>20.36133</v>
@@ -3430,10 +3424,10 @@
         <v>105.909392</v>
       </c>
       <c r="G23" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="H23" s="7" t="s">
         <v>181</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>182</v>
       </c>
       <c r="I23" s="9">
         <v>34000.0</v>
@@ -3445,7 +3439,7 @@
         <v>7</v>
       </c>
       <c r="L23" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="M23" s="9">
         <v>420</v>
@@ -3460,7 +3454,7 @@
         <v>95.0</v>
       </c>
       <c r="Q23" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="R23" s="9">
         <v>46</v>
@@ -3493,21 +3487,21 @@
         <v>0</v>
       </c>
       <c r="AB23" s="7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="24" spans="1:28" customHeight="1" ht="26">
       <c r="A24" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>186</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>187</v>
       </c>
       <c r="E24" s="8">
         <v>20.3556</v>
@@ -3516,10 +3510,10 @@
         <v>105.91240000000001</v>
       </c>
       <c r="G24" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="H24" s="7" t="s">
         <v>188</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>189</v>
       </c>
       <c r="I24" s="9">
         <v>28000.0</v>
@@ -3531,7 +3525,7 @@
         <v>5</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="M24" s="9">
         <v>300</v>
@@ -3546,7 +3540,7 @@
         <v>91.0</v>
       </c>
       <c r="Q24" s="7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="R24" s="9">
         <v>34</v>
@@ -3579,21 +3573,21 @@
         <v>0</v>
       </c>
       <c r="AB24" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="25" spans="1:28" customHeight="1" ht="26">
       <c r="A25" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="B25" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C25" s="7" t="s">
+      <c r="D25" s="7" t="s">
         <v>194</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>195</v>
       </c>
       <c r="E25" s="8">
         <v>20.5215</v>
@@ -3602,10 +3596,10 @@
         <v>105.9284</v>
       </c>
       <c r="G25" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="H25" s="7" t="s">
         <v>196</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>197</v>
       </c>
       <c r="I25" s="9">
         <v>25000.0</v>
@@ -3617,7 +3611,7 @@
         <v>5</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="M25" s="9">
         <v>360</v>
@@ -3632,7 +3626,7 @@
         <v>94.0</v>
       </c>
       <c r="Q25" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="R25" s="9">
         <v>40</v>
@@ -3665,21 +3659,21 @@
         <v>0</v>
       </c>
       <c r="AB25" s="7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="26" spans="1:28" customHeight="1" ht="26">
       <c r="A26" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="B26" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C26" s="7" t="s">
+      <c r="D26" s="7" t="s">
         <v>202</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>203</v>
       </c>
       <c r="E26" s="8">
         <v>20.3421</v>
@@ -3688,10 +3682,10 @@
         <v>105.9234</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>205</v>
+        <v>181</v>
       </c>
       <c r="I26" s="9">
         <v>30000.0</v>
@@ -3703,7 +3697,7 @@
         <v>6</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="M26" s="9">
         <v>320</v>
@@ -3718,7 +3712,7 @@
         <v>92.5</v>
       </c>
       <c r="Q26" s="7" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="R26" s="9">
         <v>36</v>
@@ -3751,7 +3745,7 @@
         <v>0</v>
       </c>
       <c r="AB26" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -3788,326 +3782,326 @@
   <sheetData>
     <row r="1" spans="1:3" customHeight="1" ht="30">
       <c r="A1" s="10" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="3" spans="1:3" customHeight="1" ht="28">
       <c r="A3" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>210</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="4" spans="1:3" customHeight="1" ht="24">
       <c r="A4" s="11" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" spans="1:3" customHeight="1" ht="24">
       <c r="A5" s="11" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" spans="1:3" customHeight="1" ht="24">
       <c r="A6" s="11" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" spans="1:3" customHeight="1" ht="24">
       <c r="A7" s="11" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:3" customHeight="1" ht="24">
       <c r="A8" s="11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:3" customHeight="1" ht="24">
       <c r="A9" s="11" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10" spans="1:3" customHeight="1" ht="24">
       <c r="A10" s="11" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" spans="1:3" customHeight="1" ht="24">
       <c r="A11" s="11" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" spans="1:3" customHeight="1" ht="24">
       <c r="A12" s="11" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="13" spans="1:3" customHeight="1" ht="24">
       <c r="A13" s="11" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" spans="1:3" customHeight="1" ht="24">
       <c r="A14" s="11" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="15" spans="1:3" customHeight="1" ht="24">
       <c r="A15" s="11" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="16" spans="1:3" customHeight="1" ht="24">
       <c r="A16" s="11" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="17" spans="1:3" customHeight="1" ht="24">
       <c r="A17" s="11" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="18" spans="1:3" customHeight="1" ht="24">
       <c r="A18" s="11" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" spans="1:3" customHeight="1" ht="24">
       <c r="A19" s="11" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="20" spans="1:3" customHeight="1" ht="24">
       <c r="A20" s="11" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="21" spans="1:3" customHeight="1" ht="24">
       <c r="A21" s="11" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="22" spans="1:3" customHeight="1" ht="24">
       <c r="A22" s="11" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="23" spans="1:3" customHeight="1" ht="24">
       <c r="A23" s="11" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24" spans="1:3" customHeight="1" ht="24">
       <c r="A24" s="11" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="25" spans="1:3" customHeight="1" ht="24">
       <c r="A25" s="11" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="26" spans="1:3" customHeight="1" ht="24">
       <c r="A26" s="11" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="27" spans="1:3" customHeight="1" ht="24">
       <c r="A27" s="11" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="28" spans="1:3" customHeight="1" ht="24">
       <c r="A28" s="11" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="29" spans="1:3" customHeight="1" ht="24">
       <c r="A29" s="11" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="30" spans="1:3" customHeight="1" ht="24">
       <c r="A30" s="11" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="31" spans="1:3" customHeight="1" ht="24">
       <c r="A31" s="11" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -4134,18 +4128,18 @@
   <sheetData>
     <row r="1" spans="1:2" customHeight="1" ht="28">
       <c r="A1" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" spans="1:2" customHeight="1" ht="22">
       <c r="A2" s="2" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:2" customHeight="1" ht="22">
@@ -4153,41 +4147,41 @@
         <v>31</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:2" customHeight="1" ht="22">
       <c r="A4" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:2" customHeight="1" ht="22">
       <c r="A5" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" spans="1:2" customHeight="1" ht="22">
       <c r="A6" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="7" spans="1:2" customHeight="1" ht="22">
       <c r="B7" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" spans="1:2" customHeight="1" ht="22">
       <c r="B8" s="2" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" spans="1:2" customHeight="1" ht="22">
@@ -4202,37 +4196,37 @@
     </row>
     <row r="11" spans="1:2" customHeight="1" ht="22">
       <c r="B11" s="2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="12" spans="1:2" customHeight="1" ht="22">
       <c r="B12" s="2" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="13" spans="1:2" customHeight="1" ht="22">
       <c r="B13" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="14" spans="1:2" customHeight="1" ht="22">
       <c r="B14" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" spans="1:2" customHeight="1" ht="22">
       <c r="B15" s="2" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="16" spans="1:2" customHeight="1" ht="22">
       <c r="B16" s="2" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="17" spans="1:2" customHeight="1" ht="22">
       <c r="B17" s="2" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="18" spans="1:2" customHeight="1" ht="22">
@@ -4242,12 +4236,12 @@
     </row>
     <row r="19" spans="1:2" customHeight="1" ht="22">
       <c r="B19" s="2" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="20" spans="1:2" customHeight="1" ht="22">
       <c r="B20" s="2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="21" spans="1:2" customHeight="1" ht="22">
@@ -4262,17 +4256,17 @@
     </row>
     <row r="23" spans="1:2" customHeight="1" ht="22">
       <c r="B23" s="2" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="24" spans="1:2" customHeight="1" ht="22">
       <c r="B24" s="2" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="25" spans="1:2" customHeight="1" ht="22">
       <c r="B25" s="2" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="26" spans="1:2" customHeight="1" ht="22">
@@ -4282,17 +4276,17 @@
     </row>
     <row r="27" spans="1:2" customHeight="1" ht="22">
       <c r="B27" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28" spans="1:2" customHeight="1" ht="22">
       <c r="B28" s="2" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="29" spans="1:2" customHeight="1" ht="22">
       <c r="B29" s="2" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="30" spans="1:2" customHeight="1" ht="22">
@@ -4302,12 +4296,12 @@
     </row>
     <row r="31" spans="1:2" customHeight="1" ht="22">
       <c r="B31" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="32" spans="1:2" customHeight="1" ht="22">
       <c r="B32" s="2" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="33" spans="1:2" customHeight="1" ht="22">
@@ -4317,487 +4311,487 @@
     </row>
     <row r="34" spans="1:2" customHeight="1" ht="22">
       <c r="B34" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="35" spans="1:2" customHeight="1" ht="22">
       <c r="B35" s="2" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="36" spans="1:2" customHeight="1" ht="22">
       <c r="B36" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="37" spans="1:2" customHeight="1" ht="22">
       <c r="B37" s="2" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="38" spans="1:2" customHeight="1" ht="22">
       <c r="B38" s="2" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="39" spans="1:2" customHeight="1" ht="22">
       <c r="B39" s="2" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="40" spans="1:2" customHeight="1" ht="22">
       <c r="B40" s="2" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="41" spans="1:2" customHeight="1" ht="22">
       <c r="B41" s="2" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="42" spans="1:2" customHeight="1" ht="22">
       <c r="B42" s="2" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="43" spans="1:2" customHeight="1" ht="22">
       <c r="B43" s="2" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="44" spans="1:2" customHeight="1" ht="22">
       <c r="B44" s="2" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="45" spans="1:2" customHeight="1" ht="22">
       <c r="B45" s="2" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="46" spans="1:2" customHeight="1" ht="22">
       <c r="B46" s="2" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="47" spans="1:2" customHeight="1" ht="22">
       <c r="B47" s="2" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="48" spans="1:2" customHeight="1" ht="22">
       <c r="B48" s="2" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="49" spans="1:2" customHeight="1" ht="22">
       <c r="B49" s="2" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="50" spans="1:2" customHeight="1" ht="22">
       <c r="B50" s="2" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="51" spans="1:2" customHeight="1" ht="22">
       <c r="B51" s="2" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="52" spans="1:2" customHeight="1" ht="22">
       <c r="B52" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="53" spans="1:2" customHeight="1" ht="22">
       <c r="B53" s="2" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="54" spans="1:2" customHeight="1" ht="22">
       <c r="B54" s="2" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="55" spans="1:2" customHeight="1" ht="22">
       <c r="B55" s="2" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="56" spans="1:2" customHeight="1" ht="22">
       <c r="B56" s="2" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="57" spans="1:2" customHeight="1" ht="22">
       <c r="B57" s="2" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="58" spans="1:2" customHeight="1" ht="22">
       <c r="B58" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="59" spans="1:2" customHeight="1" ht="22">
       <c r="B59" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="60" spans="1:2" customHeight="1" ht="22">
       <c r="B60" s="2" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="61" spans="1:2" customHeight="1" ht="22">
       <c r="B61" s="2" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="62" spans="1:2" customHeight="1" ht="22">
       <c r="B62" s="2" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="63" spans="1:2" customHeight="1" ht="22">
       <c r="B63" s="2" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="64" spans="1:2" customHeight="1" ht="22">
       <c r="B64" s="2" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="65" spans="1:2" customHeight="1" ht="22">
       <c r="B65" s="2" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="66" spans="1:2" customHeight="1" ht="22">
       <c r="B66" s="2" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="67" spans="1:2" customHeight="1" ht="22">
       <c r="B67" s="2" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="68" spans="1:2" customHeight="1" ht="22">
       <c r="B68" s="2" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="69" spans="1:2" customHeight="1" ht="22">
       <c r="B69" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="70" spans="1:2" customHeight="1" ht="22">
       <c r="B70" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="71" spans="1:2" customHeight="1" ht="22">
       <c r="B71" s="2" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="72" spans="1:2" customHeight="1" ht="22">
       <c r="B72" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="73" spans="1:2" customHeight="1" ht="22">
       <c r="B73" s="2" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="74" spans="1:2" customHeight="1" ht="22">
       <c r="B74" s="2" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="75" spans="1:2" customHeight="1" ht="22">
       <c r="B75" s="2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="76" spans="1:2" customHeight="1" ht="22">
       <c r="B76" s="2" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="77" spans="1:2" customHeight="1" ht="22">
       <c r="B77" s="2" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="78" spans="1:2" customHeight="1" ht="22">
       <c r="B78" s="2" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="79" spans="1:2" customHeight="1" ht="22">
       <c r="B79" s="2" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="80" spans="1:2" customHeight="1" ht="22">
       <c r="B80" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="81" spans="1:2" customHeight="1" ht="22">
       <c r="B81" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="82" spans="1:2" customHeight="1" ht="22">
       <c r="B82" s="2" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="83" spans="1:2" customHeight="1" ht="22">
       <c r="B83" s="2" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="84" spans="1:2" customHeight="1" ht="22">
       <c r="B84" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="85" spans="1:2" customHeight="1" ht="22">
       <c r="B85" s="2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="86" spans="1:2" customHeight="1" ht="22">
       <c r="B86" s="2" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="87" spans="1:2" customHeight="1" ht="22">
       <c r="B87" s="2" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="88" spans="1:2" customHeight="1" ht="22">
       <c r="B88" s="2" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="89" spans="1:2" customHeight="1" ht="22">
       <c r="B89" s="2" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="90" spans="1:2" customHeight="1" ht="22">
       <c r="B90" s="2" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="91" spans="1:2" customHeight="1" ht="22">
       <c r="B91" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="92" spans="1:2" customHeight="1" ht="22">
       <c r="B92" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="93" spans="1:2" customHeight="1" ht="22">
       <c r="B93" s="2" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="94" spans="1:2" customHeight="1" ht="22">
       <c r="B94" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="95" spans="1:2" customHeight="1" ht="22">
       <c r="B95" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="96" spans="1:2" customHeight="1" ht="22">
       <c r="B96" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="97" spans="1:2" customHeight="1" ht="22">
       <c r="B97" s="2" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="98" spans="1:2" customHeight="1" ht="22">
       <c r="B98" s="2" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="99" spans="1:2" customHeight="1" ht="22">
       <c r="B99" s="2" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="100" spans="1:2" customHeight="1" ht="22">
       <c r="B100" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="101" spans="1:2" customHeight="1" ht="22">
       <c r="B101" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="102" spans="1:2" customHeight="1" ht="22">
       <c r="B102" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="103" spans="1:2" customHeight="1" ht="22">
       <c r="B103" s="2" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="104" spans="1:2" customHeight="1" ht="22">
       <c r="B104" s="2" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="105" spans="1:2" customHeight="1" ht="22">
       <c r="B105" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="106" spans="1:2" customHeight="1" ht="22">
       <c r="B106" s="2" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="107" spans="1:2" customHeight="1" ht="22">
       <c r="B107" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="108" spans="1:2" customHeight="1" ht="22">
       <c r="B108" s="2" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="109" spans="1:2" customHeight="1" ht="22">
       <c r="B109" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="110" spans="1:2" customHeight="1" ht="22">
       <c r="B110" s="2" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="111" spans="1:2" customHeight="1" ht="22">
       <c r="B111" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="112" spans="1:2" customHeight="1" ht="22">
       <c r="B112" s="2" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="113" spans="1:2" customHeight="1" ht="22">
       <c r="B113" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="114" spans="1:2" customHeight="1" ht="22">
       <c r="B114" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="115" spans="1:2" customHeight="1" ht="22">
       <c r="B115" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="116" spans="1:2" customHeight="1" ht="22">
       <c r="B116" s="2" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="117" spans="1:2" customHeight="1" ht="22">
       <c r="B117" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="118" spans="1:2" customHeight="1" ht="22">
       <c r="B118" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="119" spans="1:2" customHeight="1" ht="22">
       <c r="B119" s="2" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="120" spans="1:2" customHeight="1" ht="22">
       <c r="B120" s="2" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="121" spans="1:2" customHeight="1" ht="22">
       <c r="B121" s="2" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="122" spans="1:2" customHeight="1" ht="22">
       <c r="B122" s="2" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="123" spans="1:2" customHeight="1" ht="22">
       <c r="B123" s="2" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="124" spans="1:2" customHeight="1" ht="22">
       <c r="B124" s="2" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="125" spans="1:2" customHeight="1" ht="22">
       <c r="B125" s="2" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="126" spans="1:2" customHeight="1" ht="22">
       <c r="B126" s="2" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="127" spans="1:2" customHeight="1" ht="22">
       <c r="B127" s="2" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="128" spans="1:2" customHeight="1" ht="22">
       <c r="B128" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="129" spans="1:2" customHeight="1" ht="22">
       <c r="B129" s="2" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="130" spans="1:2" customHeight="1" ht="22">
       <c r="B130" s="2" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(gis): chuan hoa thong tin xa phuong, dia chi va toa do GPS 23 truong GDNN khop 100% ranh gioi hanh chinh moi
</commit_message>
<xml_diff>
--- a/Tong_hop_truong_GDNN_tinh_Ninh_Binh_moi_2026.xlsx
+++ b/Tong_hop_truong_GDNN_tinh_Ninh_Binh_moi_2026.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="385">
   <si>
     <t>TỔNG HỢP DANH SÁCH 23 CƠ SỞ GIÁO DỤC NGHỀ NGHIỆP TỈNH NINH BÌNH (28 CỘT CHUẨN ADMIN)</t>
   </si>
@@ -139,10 +139,10 @@
     <t>Trường Cao đẳng Y tế tỉnh Ninh Bình</t>
   </si>
   <si>
-    <t>Phường Nam Thành</t>
-  </si>
-  <si>
-    <t>Số 293 Đường Hải Thượng Lãn Ông, Phường Phúc Thành, TP. Ninh Bình</t>
+    <t>Phường Hoa Lư</t>
+  </si>
+  <si>
+    <t>Số 293 Đường Hải Thượng Lãn Ông, Phường Hoa Lư, Tỉnh Ninh Bình</t>
   </si>
   <si>
     <t>0229 387 1042</t>
@@ -166,7 +166,7 @@
     <t>Phường Nam Định</t>
   </si>
   <si>
-    <t>Đường Trần Huy Liệu, Phường Năng Tĩnh, TP. Nam Định</t>
+    <t>Đường Trần Huy Liệu, Phường Nam Định, Tỉnh Ninh Bình</t>
   </si>
   <si>
     <t>0228 384 9234</t>
@@ -187,10 +187,7 @@
     <t>Trường Cao đẳng nghề LiLaMa 1</t>
   </si>
   <si>
-    <t>Phường Hoa Lư</t>
-  </si>
-  <si>
-    <t>Đường Lê Hồng Phong, Phường Hoa Lư, TP. Ninh Bình</t>
+    <t>Phường Hoa Lư, Tỉnh Ninh Bình</t>
   </si>
   <si>
     <t>0917 620 019</t>
@@ -238,7 +235,7 @@
     <t>Phường Trường Thi</t>
   </si>
   <si>
-    <t>Km6, Quốc lộ 10, Phường Trường Thi</t>
+    <t>Km6, Quốc lộ 10, Phường Trường Thi, Tỉnh Ninh Bình</t>
   </si>
   <si>
     <t>0983 703 936</t>
@@ -259,7 +256,7 @@
     <t>Trường Cao đẳng Xây dựng Nam Định</t>
   </si>
   <si>
-    <t>Quốc lộ 10, Phường Lộc Vượng, TP. Nam Định</t>
+    <t>Quốc lộ 10, Phường Nam Định, Tỉnh Ninh Bình</t>
   </si>
   <si>
     <t>0912 180 984</t>
@@ -280,10 +277,10 @@
     <t>Trường Cao đẳng Công nghệ, Kinh tế và Chế biến lâm sản</t>
   </si>
   <si>
-    <t>Thị trấn Ba Sao</t>
-  </si>
-  <si>
-    <t>Thị trấn Ba Sao, Huyện Kim Bảng, Tỉnh Hà Nam</t>
+    <t>Phường Tam Chúc</t>
+  </si>
+  <si>
+    <t>Phường Tam Chúc, Tỉnh Ninh Bình</t>
   </si>
   <si>
     <t>0226 385 4123</t>
@@ -307,7 +304,7 @@
     <t>Phường Phủ Lý</t>
   </si>
   <si>
-    <t>Số 136 đường Quy Lưu, Phường Minh Khai, TP. Phủ Lý, Tỉnh Hà Nam</t>
+    <t>Số 136 Đường Quy Lưu, Phường Phủ Lý, Tỉnh Ninh Bình</t>
   </si>
   <si>
     <t>0226 385 2772</t>
@@ -328,562 +325,550 @@
     <t>Trường Cao đẳng Cơ điện Thủy lợi Bắc Bộ (Phân hiệu tại tỉnh Ninh Bình)</t>
   </si>
   <si>
+    <t>Tổ 4, Phường Phủ Lý, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0226 385 2769</t>
+  </si>
+  <si>
+    <t>https://mwc.edu.vn/</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: ThS. Phạm Gia Điệp</t>
+  </si>
+  <si>
+    <t>Công nghệ KT Tài nguyên nước:150; Điện công nghiệp:150; Cấp thoát nước:120; Vận hành trạm bơm điện:100; Tin học ứng dụng:80</t>
+  </si>
+  <si>
+    <t>Công ty Khai thác CTTL Bắc Nam Hà:Đào tạo trạm bơm &amp; thủy lợi; Công ty CP Nước sạch Hà Nam:Tuyển dụng kỹ sư cấp thoát nước</t>
+  </si>
+  <si>
+    <t>Trường Cao đẳng nghề Số 20 - BQP</t>
+  </si>
+  <si>
+    <t>Số 126C Trần Đăng Ninh, Phường Nam Định, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0228 383 4465</t>
+  </si>
+  <si>
+    <t>https://caodang20.edu.vn/</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: Trần Quang Dũng</t>
+  </si>
+  <si>
+    <t>Công nghệ ô tô:300; Điện tử công nghiệp:200; KT Lắp đặt điện trong CN:200; Vận hành máy thi công nền:150; May thời trang:120</t>
+  </si>
+  <si>
+    <t>Tổng công ty Kinh tế Kỹ thuật Công nghiệp Quốc phòng:Tuyển dụng kỹ thuật viên cơ khí &amp; ô tô</t>
+  </si>
+  <si>
+    <t>Trường Cao đẳng FPT Polytechnic cơ sở Hà Nam</t>
+  </si>
+  <si>
+    <t>Phường Hà Nam</t>
+  </si>
+  <si>
+    <t>Đường Độc Lập, KĐT Đại học Nam Cao, Phường Hà Nam, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0226 730 0999</t>
+  </si>
+  <si>
+    <t>https://caodang.fpt.edu.vn/</t>
+  </si>
+  <si>
+    <t>Giám đốc: Vũ Chí Thành</t>
+  </si>
+  <si>
+    <t>Lập trình máy tính:400; Thiết kế đồ họa:300; Quản lý vận tải và dịch vụ logistics:250; Quản trị kinh doanh:200; Tiếng Trung Quốc:150</t>
+  </si>
+  <si>
+    <t>Tập đoàn FPT:Bao tiêu việc làm ngành CNTT; Công ty FPT Software:Thực tập dự án phần mềm</t>
+  </si>
+  <si>
+    <t>Trường Cao đẳng Công nghiệp Dệt - May Nam Định</t>
+  </si>
+  <si>
+    <t>Số 6 Đường Hoàng Diệu, Phường Nam Định, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0228 384 8562</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: ThS. Lê Thị Mai</t>
+  </si>
+  <si>
+    <t>Công nghệ may:200; May thời trang:150; Thiết kế thời trang:100; Sửa chữa thiết bị may:80</t>
+  </si>
+  <si>
+    <t>Tổng công ty CP Dệt may Nam Định:Hợp tác đào tạo chuỗi cung ứng dệt may</t>
+  </si>
+  <si>
+    <t>Trường Cao đẳng Sư phạm Nam Định</t>
+  </si>
+  <si>
+    <t>Số 84 Đường Lê Hồng Phong, Phường Nam Định, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0228 384 9452</t>
+  </si>
+  <si>
+    <t>https://cdspnd.edu.vn/</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: TS. Trần Duy Hưng</t>
+  </si>
+  <si>
+    <t>Giáo dục Mầm non:250; Giáo dục Tiểu học:200; Sư phạm Tiếng Anh:100</t>
+  </si>
+  <si>
+    <t>Hệ thống Trường Mầm non Quốc tế Vinschool:Tuyển dụng giáo viên mầm non</t>
+  </si>
+  <si>
+    <t>Trường Trung cấp Giao thông vận tải tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>Trung cấp</t>
+  </si>
+  <si>
+    <t>Quốc lộ 10, Phường Trường Thi, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0985 453 868</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/TTSHLXNB/</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: Phạm Quang Thể</t>
+  </si>
+  <si>
+    <t>Công nghệ ô tô:150; Điện công nghiệp:120; Kế toán doanh nghiệp:80; Sửa chữa máy tính:50</t>
+  </si>
+  <si>
+    <t>Công ty CP Vận tải Ninh Bình:Tuyển dụng kỹ thuật viên bảo dưỡng ô tô</t>
+  </si>
+  <si>
+    <t>Trường Trung cấp Công nghệ số 8 Nam Định</t>
+  </si>
+  <si>
+    <t>Phường Vị Khê</t>
+  </si>
+  <si>
+    <t>Tổ dân phố Đông Đồng Ngãi, Phường Vị Khê, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0913 517 988</t>
+  </si>
+  <si>
+    <t>https://www.truongtccn8nd.edu.vn/</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: Nguyễn Chí Thuấn</t>
+  </si>
+  <si>
+    <t>Bảo trì và sửa chữa ô tô:120; Điện công nghiệp:100; Công nghệ thông tin:80; Hàn:60; May thời trang:50</t>
+  </si>
+  <si>
+    <t>Công ty TNHH Cơ khí Tân Á:Hợp tác đào tạo nghề hàn &amp; cơ khí</t>
+  </si>
+  <si>
+    <t>Trường Trung cấp Kỹ thuật - Du lịch Công đoàn Ninh Bình</t>
+  </si>
+  <si>
+    <t>Đường Triệu Việt Vương, Phường Hoa Lư, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0988 119 197</t>
+  </si>
+  <si>
+    <t>http://tccdnb.edu.vn/</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: Dương Mạnh Hiền</t>
+  </si>
+  <si>
+    <t>Hướng dẫn du lịch:150; Quản trị khách sạn:120; Nghiệp vụ nhà hàng:100; Kỹ thuật chế biến món ăn:100; May thời trang:80</t>
+  </si>
+  <si>
+    <t>Khu Du lịch Sinh thái Tràng An:Tiếp nhận thực tập nghiệp vụ du lịch &amp; nhà hàng; Khách sạn Hoàng Sơn Peace:Hợp tác đào tạo buồng phòng</t>
+  </si>
+  <si>
+    <t>Trường Trung cấp Đại Lâm</t>
+  </si>
+  <si>
+    <t>Phường Thiên Trường</t>
+  </si>
+  <si>
+    <t>Quốc lộ 10, Phường Thiên Trường, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0918 843 843</t>
+  </si>
+  <si>
+    <t>https://truongtrungcapdailam.edu.vn/</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: Trần Thọ Hiền</t>
+  </si>
+  <si>
+    <t>Công nghệ ô tô:150; May thời trang:120</t>
+  </si>
+  <si>
+    <t>Công ty CP Ô tô Nam Định:Thực tập sinh kỹ thuật ô tô</t>
+  </si>
+  <si>
+    <t>Trường Trung cấp Y - Dược Tôn Thất Tùng</t>
+  </si>
+  <si>
+    <t>Phường Nam Định, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0228 368 6868</t>
+  </si>
+  <si>
+    <t>https://truongyduoctonthattung.com.vn/</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: BS. Tôn Thất Hưng</t>
+  </si>
+  <si>
+    <t>Y Sỹ:120; Y học cổ truyền:80; Dược:100; Điều Dưỡng:100; Kỹ thuật xét nghiệm y học:50</t>
+  </si>
+  <si>
+    <t>Bệnh viện Đa khoa tỉnh Nam Định:Thực tập lâm sàng sinh viên y khoa</t>
+  </si>
+  <si>
+    <t>Trường Trung cấp nghề Quốc tế</t>
+  </si>
+  <si>
+    <t>Xã Gia Trấn</t>
+  </si>
+  <si>
+    <t>Km10, Quốc lộ 1A, Xã Gia Trấn, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0913 583 517</t>
+  </si>
+  <si>
+    <t>https://ivsedu.vn/</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: Trần Minh Chất</t>
+  </si>
+  <si>
+    <t>Tiếng Trung Quốc:150; Công nghệ thông tin:120; Kỹ thuật Chế biến món ăn:100; Điện công nghiệp:100; May thời trang:80</t>
+  </si>
+  <si>
+    <t>Công ty TNHH Greatstar Ninh Bình:Cung ứng nhân lực biết tiếng Trung; KCN Gián Khẩu:Tuyển dụng kỹ thuật viên điện</t>
+  </si>
+  <si>
+    <t>Trường Trung cấp nghề Giao thông - Xây dựng Việt Úc</t>
+  </si>
+  <si>
+    <t>Xã Gia Trấn, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0229 386 8899</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/vietuchanam/</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: ThS. Nguyễn Văn Úc</t>
+  </si>
+  <si>
+    <t>Vận hành máy thi công nền:120; Kỹ thuật xây dựng:100; Lái xe ô tô các hạng:150</t>
+  </si>
+  <si>
+    <t>Công ty CP Đầu tư Xây dựng Ninh Bình:Thực tập thi công công trình giao thông</t>
+  </si>
+  <si>
+    <t>Trường Trung cấp Y - Dược Hà Nam</t>
+  </si>
+  <si>
+    <t>Đường Lê Duẩn, Phường Phủ Lý, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0226 388 3456</t>
+  </si>
+  <si>
+    <t>https://yduochanam.blogspot.com/</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: DS. Trần Thị Minh</t>
+  </si>
+  <si>
+    <t>Y Sỹ:120; Dược Sỹ Trung cấp:100; Điều Dưỡng:100; Hộ sinh:60</t>
+  </si>
+  <si>
+    <t>Bệnh viện Đa khoa tỉnh Hà Nam:Thực tập hộ sinh và y sỹ</t>
+  </si>
+  <si>
+    <t>Trường Trung cấp nghề Kỹ thuật cao Quốc tế</t>
+  </si>
+  <si>
+    <t>Khu Công nghiệp Gián Khẩu, Xã Gia Trấn, Tỉnh Ninh Bình</t>
+  </si>
+  <si>
+    <t>0229 383 6789</t>
+  </si>
+  <si>
+    <t>Hiệu trưởng: ThS. Đỗ Văn Cương</t>
+  </si>
+  <si>
+    <t>Hàn công nghệ cao:120; Điện công nghiệp:100; Cắt gọt kim loại CNC:80; Kỹ thuật ô tô:80</t>
+  </si>
+  <si>
+    <t>Công ty TNHH Mcnex Vina:Hợp tác đào tạo kỹ thuật viên tự động hóa</t>
+  </si>
+  <si>
+    <t>BẢNG GIẢI THÍCH QUY ƯỚC CỘT VÀ ĐỊNH DẠNG DỮ LIỆU (ĐỒNG BỘ 5 TAB ADMIN)</t>
+  </si>
+  <si>
+    <t>Cột</t>
+  </si>
+  <si>
+    <t>Tên trường thông tin</t>
+  </si>
+  <si>
+    <t>Quy ước nhập liệu &amp; Giá trị hợp lệ</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Bắt buộc. Tên đầy đủ của cơ sở giáo dục</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Bắt buộc. Chọn từ danh sách xổ xuống (Đại học, Cao đẳng, Trung cấp, GDTX...)</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Chọn từ danh sách xổ xuống (129 xã/phường có sẵn trong sheet Danh_Muc)</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Số nhà, tên đường, khu đô thị</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>Tọa độ GPS thập phân WGS84 (VD: 20.2605)</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>Tọa độ GPS thập phân WGS84 (VD: 105.9750)</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>Số hotline hoặc điện thoại bàn liên hệ</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>Địa chỉ website hoặc cổng thông tin (VD: https://cdyteninhbinh.edu.vn)</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>Tổng diện tích mặt bằng khuôn viên trường (m²)</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>Tổng số phòng học lý thuyết và giảng đường</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>Tổng số xưởng kỹ thuật, phòng thực hành, phòng thí nghiệm</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Cú pháp: Chức vụ: Họ tên; Chức vụ 2: Họ tên 2 (VD: Hiệu trưởng: PGS.TS. Vũ Văn Hùng; Phó Hiệu trưởng: TS. Nguyễn Văn A)</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>Chỉ tiêu / số lượng học sinh, sinh viên tuyển sinh mới mỗi năm</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Tổng quy mô học sinh/sinh viên đang theo học hiện tại</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>Số lượng học sinh/sinh viên ra trường mỗi năm</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Tỷ lệ sinh viên có việc làm sau tốt nghiệp (VD: 94.5)</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>Cú pháp: Tên ngành:Chỉ tiêu, cách nhau bằng dấu chấm phẩy ;</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>Tổng số cán bộ, giáo viên, giảng viên hiện có</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Tổng chỉ tiêu biên chế Sở / Bộ giao</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>Số lượng cán bộ giảng dạy còn thiếu so với định biên</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>Số lượng cán bộ giảng dạy dôi dư (nếu có)</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>Số giảng viên đạt tiêu chuẩn Hạng I / Loại 1</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>Số giảng viên đạt tiêu chuẩn Hạng II / Loại 2</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Số giảng viên tiêu chuẩn Hạng III</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Số lượng cán bộ có học vị Tiến sĩ</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>Số lượng cán bộ có học vị Thạc sĩ</t>
+  </si>
+  <si>
+    <t>AA</t>
+  </si>
+  <si>
+    <t>Số lượng cán bộ có học hàm Giáo sư, Phó Giáo sư</t>
+  </si>
+  <si>
+    <t>AB</t>
+  </si>
+  <si>
+    <t>Cú pháp: Tên DN:Nội dung hợp tác, cách nhau bằng dấu chấm phẩy ;</t>
+  </si>
+  <si>
+    <t>Danh sách Cấp học</t>
+  </si>
+  <si>
+    <t>Danh sách Xã / Phường (129 đơn vị)</t>
+  </si>
+  <si>
+    <t>Đại học</t>
+  </si>
+  <si>
+    <t>Phường Châu Sơn</t>
+  </si>
+  <si>
+    <t>Phường Duy Hà</t>
+  </si>
+  <si>
+    <t>Phường Duy Tân</t>
+  </si>
+  <si>
+    <t>GDTX</t>
+  </si>
+  <si>
+    <t>Phường Duy Tiên</t>
+  </si>
+  <si>
+    <t>GDTX - GDNN</t>
+  </si>
+  <si>
+    <t>Phường Đông A</t>
+  </si>
+  <si>
+    <t>Phường Đông Hoa Lư</t>
+  </si>
+  <si>
+    <t>Phường Đồng Văn</t>
+  </si>
+  <si>
+    <t>Phường Hồng Quang</t>
+  </si>
+  <si>
+    <t>Phường Kim Bảng</t>
+  </si>
+  <si>
+    <t>Phường Kim Thanh</t>
+  </si>
+  <si>
+    <t>Phường Lê Hồ</t>
+  </si>
+  <si>
+    <t>Phường Liêm Tuyền</t>
+  </si>
+  <si>
+    <t>Phường Lý Thường Kiệt</t>
+  </si>
+  <si>
+    <t>Phường Mỹ Lộc</t>
+  </si>
+  <si>
+    <t>Phường Nam Hoa Lư</t>
+  </si>
+  <si>
+    <t>Phường Nguyễn Úy</t>
+  </si>
+  <si>
     <t>Phường Phù Vân</t>
-  </si>
-  <si>
-    <t>Xã Phù Vân, TP. Phủ Lý, Tỉnh Hà Nam</t>
-  </si>
-  <si>
-    <t>0226 385 2769</t>
-  </si>
-  <si>
-    <t>https://mwc.edu.vn/</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: ThS. Phạm Gia Điệp</t>
-  </si>
-  <si>
-    <t>Công nghệ KT Tài nguyên nước:150; Điện công nghiệp:150; Cấp thoát nước:120; Vận hành trạm bơm điện:100; Tin học ứng dụng:80</t>
-  </si>
-  <si>
-    <t>Công ty Khai thác CTTL Bắc Nam Hà:Đào tạo trạm bơm &amp; thủy lợi; Công ty CP Nước sạch Hà Nam:Tuyển dụng kỹ sư cấp thoát nước</t>
-  </si>
-  <si>
-    <t>Trường Cao đẳng nghề Số 20 - BQP</t>
-  </si>
-  <si>
-    <t>Số 126C Trần Đăng Ninh, Phường Nam Định</t>
-  </si>
-  <si>
-    <t>0228 383 4465</t>
-  </si>
-  <si>
-    <t>https://caodang20.edu.vn/</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: Trần Quang Dũng</t>
-  </si>
-  <si>
-    <t>Công nghệ ô tô:300; Điện tử công nghiệp:200; KT Lắp đặt điện trong CN:200; Vận hành máy thi công nền:150; May thời trang:120</t>
-  </si>
-  <si>
-    <t>Tổng công ty Kinh tế Kỹ thuật Công nghiệp Quốc phòng:Tuyển dụng kỹ thuật viên cơ khí &amp; ô tô</t>
-  </si>
-  <si>
-    <t>Trường Cao đẳng FPT Polytechnic cơ sở Hà Nam</t>
-  </si>
-  <si>
-    <t>Phường Hà Nam</t>
-  </si>
-  <si>
-    <t>Đường Độc Lập, KĐT Đại học Nam Cao, Thị xã Duy Tiên, Tỉnh Hà Nam</t>
-  </si>
-  <si>
-    <t>0226 730 0999</t>
-  </si>
-  <si>
-    <t>https://caodang.fpt.edu.vn/</t>
-  </si>
-  <si>
-    <t>Giám đốc: Vũ Chí Thành</t>
-  </si>
-  <si>
-    <t>Lập trình máy tính:400; Thiết kế đồ họa:300; Quản lý vận tải và dịch vụ logistics:250; Quản trị kinh doanh:200; Tiếng Trung Quốc:150</t>
-  </si>
-  <si>
-    <t>Tập đoàn FPT:Bao tiêu việc làm ngành CNTT; Công ty FPT Software:Thực tập dự án phần mềm</t>
-  </si>
-  <si>
-    <t>Trường Cao đẳng Công nghiệp Dệt - May Nam Định</t>
-  </si>
-  <si>
-    <t>Số 1 Đường Tô Hiến Thành, Phường Trường Thi, TP. Nam Định</t>
-  </si>
-  <si>
-    <t>0228 384 8562</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: ThS. Lê Thị Mai</t>
-  </si>
-  <si>
-    <t>Công nghệ may:200; May thời trang:150; Thiết kế thời trang:100; Sửa chữa thiết bị may:80</t>
-  </si>
-  <si>
-    <t>Tổng công ty CP Dệt may Nam Định:Hợp tác đào tạo chuỗi cung ứng dệt may</t>
-  </si>
-  <si>
-    <t>Trường Cao đẳng Sư phạm Nam Định</t>
-  </si>
-  <si>
-    <t>Số 84 Đường Lê Hồng Phong, Phường Vị Xuyên, TP. Nam Định</t>
-  </si>
-  <si>
-    <t>0228 384 9452</t>
-  </si>
-  <si>
-    <t>https://cdspnd.edu.vn/</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: TS. Trần Duy Hưng</t>
-  </si>
-  <si>
-    <t>Giáo dục Mầm non:250; Giáo dục Tiểu học:200; Sư phạm Tiếng Anh:100</t>
-  </si>
-  <si>
-    <t>Hệ thống Trường Mầm non Quốc tế Vinschool:Tuyển dụng giáo viên mầm non</t>
-  </si>
-  <si>
-    <t>Trường Trung cấp Giao thông vận tải tỉnh Ninh Bình</t>
-  </si>
-  <si>
-    <t>Trung cấp</t>
-  </si>
-  <si>
-    <t>Km 110 + 700, Quốc lộ 10, Phường Trường Thi</t>
-  </si>
-  <si>
-    <t>0985 453 868</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/TTSHLXNB/</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: Phạm Quang Thể</t>
-  </si>
-  <si>
-    <t>Công nghệ ô tô:150; Điện công nghiệp:120; Kế toán doanh nghiệp:80; Sửa chữa máy tính:50</t>
-  </si>
-  <si>
-    <t>Công ty CP Vận tải Ninh Bình:Tuyển dụng kỹ thuật viên bảo dưỡng ô tô</t>
-  </si>
-  <si>
-    <t>Trường Trung cấp Công nghệ số 8 Nam Định</t>
-  </si>
-  <si>
-    <t>Phường Vị Khê</t>
-  </si>
-  <si>
-    <t>Phường Vị Khê, Tỉnh Ninh Bình</t>
-  </si>
-  <si>
-    <t>0913 517 988</t>
-  </si>
-  <si>
-    <t>https://www.truongtccn8nd.edu.vn/</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: Nguyễn Chí Thuấn</t>
-  </si>
-  <si>
-    <t>Bảo trì và sửa chữa ô tô:120; Điện công nghiệp:100; Công nghệ thông tin:80; Hàn:60; May thời trang:50</t>
-  </si>
-  <si>
-    <t>Công ty TNHH Cơ khí Tân Á:Hợp tác đào tạo nghề hàn &amp; cơ khí</t>
-  </si>
-  <si>
-    <t>Trường Trung cấp Kỹ thuật - Du lịch Công đoàn Ninh Bình</t>
-  </si>
-  <si>
-    <t>Phường Bích Đào</t>
-  </si>
-  <si>
-    <t>Đường Triệu Việt Vương, Phường Bích Đào, TP. Ninh Bình</t>
-  </si>
-  <si>
-    <t>0988 119 197</t>
-  </si>
-  <si>
-    <t>http://tccdnb.edu.vn/</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: Dương Mạnh Hiền</t>
-  </si>
-  <si>
-    <t>Hướng dẫn du lịch:150; Quản trị khách sạn:120; Nghiệp vụ nhà hàng:100; Kỹ thuật chế biến món ăn:100; May thời trang:80</t>
-  </si>
-  <si>
-    <t>Khu Du lịch Sinh thái Tràng An:Tiếp nhận thực tập nghiệp vụ du lịch &amp; nhà hàng; Khách sạn Hoàng Sơn Peace:Hợp tác đào tạo buồng phòng</t>
-  </si>
-  <si>
-    <t>Trường Trung cấp Đại Lâm</t>
-  </si>
-  <si>
-    <t>Phường Thiên Trường</t>
-  </si>
-  <si>
-    <t>Quốc lộ 10, Phường Thiên Trường, Tỉnh Ninh Bình</t>
-  </si>
-  <si>
-    <t>0918 843 843</t>
-  </si>
-  <si>
-    <t>https://truongtrungcapdailam.edu.vn/</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: Trần Thọ Hiền</t>
-  </si>
-  <si>
-    <t>Công nghệ ô tô:150; May thời trang:120</t>
-  </si>
-  <si>
-    <t>Công ty CP Ô tô Nam Định:Thực tập sinh kỹ thuật ô tô</t>
-  </si>
-  <si>
-    <t>Trường Trung cấp Y - Dược Tôn Thất Tùng</t>
-  </si>
-  <si>
-    <t>Phường Lộc Vượng, TP. Nam Định</t>
-  </si>
-  <si>
-    <t>0228 368 6868</t>
-  </si>
-  <si>
-    <t>https://truongyduoctonthattung.com.vn/</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: BS. Tôn Thất Hưng</t>
-  </si>
-  <si>
-    <t>Y Sỹ:120; Y học cổ truyền:80; Dược:100; Điều Dưỡng:100; Kỹ thuật xét nghiệm y học:50</t>
-  </si>
-  <si>
-    <t>Bệnh viện Đa khoa tỉnh Nam Định:Thực tập lâm sàng sinh viên y khoa</t>
-  </si>
-  <si>
-    <t>Trường Trung cấp nghề Quốc tế</t>
-  </si>
-  <si>
-    <t>Xã Gia Trấn</t>
-  </si>
-  <si>
-    <t>Km10, Quốc lộ 1A, Xã Gia Trấn, Tỉnh Ninh Bình</t>
-  </si>
-  <si>
-    <t>0913 583 517</t>
-  </si>
-  <si>
-    <t>https://ivsedu.vn/</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: Trần Minh Chất</t>
-  </si>
-  <si>
-    <t>Tiếng Trung Quốc:150; Công nghệ thông tin:120; Kỹ thuật Chế biến món ăn:100; Điện công nghiệp:100; May thời trang:80</t>
-  </si>
-  <si>
-    <t>Công ty TNHH Greatstar Ninh Bình:Cung ứng nhân lực biết tiếng Trung; KCN Gián Khẩu:Tuyển dụng kỹ thuật viên điện</t>
-  </si>
-  <si>
-    <t>Trường Trung cấp nghề Giao thông - Xây dựng Việt Úc</t>
-  </si>
-  <si>
-    <t>Xã Gia Trấn, Huyện Gia Viễn, Tỉnh Ninh Bình</t>
-  </si>
-  <si>
-    <t>0229 386 8899</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/vietuchanam/</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: ThS. Nguyễn Văn Úc</t>
-  </si>
-  <si>
-    <t>Vận hành máy thi công nền:120; Kỹ thuật xây dựng:100; Lái xe ô tô các hạng:150</t>
-  </si>
-  <si>
-    <t>Công ty CP Đầu tư Xây dựng Ninh Bình:Thực tập thi công công trình giao thông</t>
-  </si>
-  <si>
-    <t>Trường Trung cấp Y - Dược Hà Nam</t>
-  </si>
-  <si>
-    <t>Phường Liêm Chính</t>
-  </si>
-  <si>
-    <t>Đường Lê Duẩn, Phường Liêm Chính, TP. Phủ Lý, Tỉnh Hà Nam</t>
-  </si>
-  <si>
-    <t>0226 388 3456</t>
-  </si>
-  <si>
-    <t>https://yduochanam.blogspot.com/</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: DS. Trần Thị Minh</t>
-  </si>
-  <si>
-    <t>Y Sỹ:120; Dược Sỹ Trung cấp:100; Điều Dưỡng:100; Hộ sinh:60</t>
-  </si>
-  <si>
-    <t>Bệnh viện Đa khoa tỉnh Hà Nam:Thực tập hộ sinh và y sỹ</t>
-  </si>
-  <si>
-    <t>Trường Trung cấp nghề Kỹ thuật cao Quốc tế</t>
-  </si>
-  <si>
-    <t>Xã Gia Tân</t>
-  </si>
-  <si>
-    <t>Khu Công nghiệp Gián Khẩu, Huyện Gia Viễn, Tỉnh Ninh Bình</t>
-  </si>
-  <si>
-    <t>0229 383 6789</t>
-  </si>
-  <si>
-    <t>Hiệu trưởng: ThS. Đỗ Văn Cương</t>
-  </si>
-  <si>
-    <t>Hàn công nghệ cao:120; Điện công nghiệp:100; Cắt gọt kim loại CNC:80; Kỹ thuật ô tô:80</t>
-  </si>
-  <si>
-    <t>Công ty TNHH Mcnex Vina:Hợp tác đào tạo kỹ thuật viên tự động hóa</t>
-  </si>
-  <si>
-    <t>BẢNG GIẢI THÍCH QUY ƯỚC CỘT VÀ ĐỊNH DẠNG DỮ LIỆU (ĐỒNG BỘ 5 TAB ADMIN)</t>
-  </si>
-  <si>
-    <t>Cột</t>
-  </si>
-  <si>
-    <t>Tên trường thông tin</t>
-  </si>
-  <si>
-    <t>Quy ước nhập liệu &amp; Giá trị hợp lệ</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Bắt buộc. Tên đầy đủ của cơ sở giáo dục</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>Bắt buộc. Chọn từ danh sách xổ xuống (Đại học, Cao đẳng, Trung cấp, GDTX...)</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>Chọn từ danh sách xổ xuống (129 xã/phường có sẵn trong sheet Danh_Muc)</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>Số nhà, tên đường, khu đô thị</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>Tọa độ GPS thập phân WGS84 (VD: 20.2605)</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>Tọa độ GPS thập phân WGS84 (VD: 105.9750)</t>
-  </si>
-  <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>Số hotline hoặc điện thoại bàn liên hệ</t>
-  </si>
-  <si>
-    <t>H</t>
-  </si>
-  <si>
-    <t>Địa chỉ website hoặc cổng thông tin (VD: https://cdyteninhbinh.edu.vn)</t>
-  </si>
-  <si>
-    <t>I</t>
-  </si>
-  <si>
-    <t>Tổng diện tích mặt bằng khuôn viên trường (m²)</t>
-  </si>
-  <si>
-    <t>J</t>
-  </si>
-  <si>
-    <t>Tổng số phòng học lý thuyết và giảng đường</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
-  <si>
-    <t>Tổng số xưởng kỹ thuật, phòng thực hành, phòng thí nghiệm</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>Cú pháp: Chức vụ: Họ tên; Chức vụ 2: Họ tên 2 (VD: Hiệu trưởng: PGS.TS. Vũ Văn Hùng; Phó Hiệu trưởng: TS. Nguyễn Văn A)</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>Chỉ tiêu / số lượng học sinh, sinh viên tuyển sinh mới mỗi năm</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>Tổng quy mô học sinh/sinh viên đang theo học hiện tại</t>
-  </si>
-  <si>
-    <t>O</t>
-  </si>
-  <si>
-    <t>Số lượng học sinh/sinh viên ra trường mỗi năm</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t>Tỷ lệ sinh viên có việc làm sau tốt nghiệp (VD: 94.5)</t>
-  </si>
-  <si>
-    <t>Q</t>
-  </si>
-  <si>
-    <t>Cú pháp: Tên ngành:Chỉ tiêu, cách nhau bằng dấu chấm phẩy ;</t>
-  </si>
-  <si>
-    <t>R</t>
-  </si>
-  <si>
-    <t>Tổng số cán bộ, giáo viên, giảng viên hiện có</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>Tổng chỉ tiêu biên chế Sở / Bộ giao</t>
-  </si>
-  <si>
-    <t>T</t>
-  </si>
-  <si>
-    <t>Số lượng cán bộ giảng dạy còn thiếu so với định biên</t>
-  </si>
-  <si>
-    <t>U</t>
-  </si>
-  <si>
-    <t>Số lượng cán bộ giảng dạy dôi dư (nếu có)</t>
-  </si>
-  <si>
-    <t>V</t>
-  </si>
-  <si>
-    <t>Số giảng viên đạt tiêu chuẩn Hạng I / Loại 1</t>
-  </si>
-  <si>
-    <t>W</t>
-  </si>
-  <si>
-    <t>Số giảng viên đạt tiêu chuẩn Hạng II / Loại 2</t>
-  </si>
-  <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>Số giảng viên tiêu chuẩn Hạng III</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>Số lượng cán bộ có học vị Tiến sĩ</t>
-  </si>
-  <si>
-    <t>Z</t>
-  </si>
-  <si>
-    <t>Số lượng cán bộ có học vị Thạc sĩ</t>
-  </si>
-  <si>
-    <t>AA</t>
-  </si>
-  <si>
-    <t>Số lượng cán bộ có học hàm Giáo sư, Phó Giáo sư</t>
-  </si>
-  <si>
-    <t>AB</t>
-  </si>
-  <si>
-    <t>Cú pháp: Tên DN:Nội dung hợp tác, cách nhau bằng dấu chấm phẩy ;</t>
-  </si>
-  <si>
-    <t>Danh sách Cấp học</t>
-  </si>
-  <si>
-    <t>Danh sách Xã / Phường (129 đơn vị)</t>
-  </si>
-  <si>
-    <t>Đại học</t>
-  </si>
-  <si>
-    <t>Phường Châu Sơn</t>
-  </si>
-  <si>
-    <t>Phường Duy Hà</t>
-  </si>
-  <si>
-    <t>Phường Duy Tân</t>
-  </si>
-  <si>
-    <t>GDTX</t>
-  </si>
-  <si>
-    <t>Phường Duy Tiên</t>
-  </si>
-  <si>
-    <t>GDTX - GDNN</t>
-  </si>
-  <si>
-    <t>Phường Đông A</t>
-  </si>
-  <si>
-    <t>Phường Đông Hoa Lư</t>
-  </si>
-  <si>
-    <t>Phường Đồng Văn</t>
-  </si>
-  <si>
-    <t>Phường Hồng Quang</t>
-  </si>
-  <si>
-    <t>Phường Kim Bảng</t>
-  </si>
-  <si>
-    <t>Phường Kim Thanh</t>
-  </si>
-  <si>
-    <t>Phường Lê Hồ</t>
-  </si>
-  <si>
-    <t>Phường Liêm Tuyền</t>
-  </si>
-  <si>
-    <t>Phường Lý Thường Kiệt</t>
-  </si>
-  <si>
-    <t>Phường Mỹ Lộc</t>
-  </si>
-  <si>
-    <t>Phường Nam Hoa Lư</t>
-  </si>
-  <si>
-    <t>Phường Nguyễn Úy</t>
-  </si>
-  <si>
-    <t>Phường Tam Chúc</t>
   </si>
   <si>
     <t>Phường Tam Điệp</t>
@@ -2036,22 +2021,22 @@
         <v>31</v>
       </c>
       <c r="C7" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="E7" s="8">
+        <v>20.26515</v>
+      </c>
+      <c r="F7" s="8">
+        <v>105.942854</v>
+      </c>
+      <c r="G7" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="8">
-        <v>20.258751</v>
-      </c>
-      <c r="F7" s="8">
-        <v>105.97639700000001</v>
-      </c>
-      <c r="G7" s="8" t="s">
+      <c r="H7" s="7" t="s">
         <v>58</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>59</v>
       </c>
       <c r="I7" s="9">
         <v>85000.0</v>
@@ -2063,7 +2048,7 @@
         <v>16</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M7" s="9">
         <v>1100</v>
@@ -2078,7 +2063,7 @@
         <v>97.5</v>
       </c>
       <c r="Q7" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="R7" s="9">
         <v>125</v>
@@ -2111,21 +2096,21 @@
         <v>0</v>
       </c>
       <c r="AB7" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:28" customHeight="1" ht="26">
       <c r="A8" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C8" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>64</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>65</v>
       </c>
       <c r="E8" s="8">
         <v>20.161953</v>
@@ -2134,10 +2119,10 @@
         <v>105.963112</v>
       </c>
       <c r="G8" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="H8" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="I8" s="9">
         <v>92000.0</v>
@@ -2149,7 +2134,7 @@
         <v>15</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M8" s="9">
         <v>1050</v>
@@ -2164,7 +2149,7 @@
         <v>95.0</v>
       </c>
       <c r="Q8" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="R8" s="9">
         <v>118</v>
@@ -2197,33 +2182,33 @@
         <v>0</v>
       </c>
       <c r="AB8" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:28" customHeight="1" ht="26">
       <c r="A9" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C9" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="8">
+        <v>20.37461</v>
+      </c>
+      <c r="F9" s="8">
+        <v>106.134744</v>
+      </c>
+      <c r="G9" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="E9" s="8">
-        <v>20.384124</v>
-      </c>
-      <c r="F9" s="8">
-        <v>106.138508</v>
-      </c>
-      <c r="G9" s="8" t="s">
+      <c r="H9" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>75</v>
       </c>
       <c r="I9" s="9">
         <v>75000.0</v>
@@ -2235,7 +2220,7 @@
         <v>14</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="M9" s="9">
         <v>850</v>
@@ -2250,7 +2235,7 @@
         <v>94.2</v>
       </c>
       <c r="Q9" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="R9" s="9">
         <v>105</v>
@@ -2283,12 +2268,12 @@
         <v>0</v>
       </c>
       <c r="AB9" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:28" customHeight="1" ht="26">
       <c r="A10" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>31</v>
@@ -2297,19 +2282,19 @@
         <v>48</v>
       </c>
       <c r="D10" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="8">
+        <v>20.444673</v>
+      </c>
+      <c r="F10" s="8">
+        <v>106.17272</v>
+      </c>
+      <c r="G10" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="E10" s="8">
-        <v>20.451005</v>
-      </c>
-      <c r="F10" s="8">
-        <v>106.17151800000001</v>
-      </c>
-      <c r="G10" s="8" t="s">
+      <c r="H10" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="I10" s="9">
         <v>65000.0</v>
@@ -2321,7 +2306,7 @@
         <v>11</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="M10" s="9">
         <v>750</v>
@@ -2336,7 +2321,7 @@
         <v>93.8</v>
       </c>
       <c r="Q10" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="R10" s="9">
         <v>92</v>
@@ -2369,21 +2354,21 @@
         <v>0</v>
       </c>
       <c r="AB10" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:28" customHeight="1" ht="26">
       <c r="A11" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C11" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>87</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>88</v>
       </c>
       <c r="E11" s="8">
         <v>20.5342</v>
@@ -2392,10 +2377,10 @@
         <v>105.8125</v>
       </c>
       <c r="G11" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="H11" s="7" t="s">
         <v>89</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="I11" s="9">
         <v>58000.0</v>
@@ -2407,7 +2392,7 @@
         <v>10</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M11" s="9">
         <v>650</v>
@@ -2422,7 +2407,7 @@
         <v>92.5</v>
       </c>
       <c r="Q11" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="R11" s="9">
         <v>78</v>
@@ -2455,21 +2440,21 @@
         <v>0</v>
       </c>
       <c r="AB11" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:28" customHeight="1" ht="26">
       <c r="A12" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>95</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>96</v>
       </c>
       <c r="E12" s="8">
         <v>20.53982</v>
@@ -2478,10 +2463,10 @@
         <v>105.91421</v>
       </c>
       <c r="G12" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="H12" s="7" t="s">
         <v>97</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>98</v>
       </c>
       <c r="I12" s="9">
         <v>45000.0</v>
@@ -2493,7 +2478,7 @@
         <v>12</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M12" s="9">
         <v>800</v>
@@ -2508,7 +2493,7 @@
         <v>95.5</v>
       </c>
       <c r="Q12" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="R12" s="9">
         <v>95</v>
@@ -2541,21 +2526,21 @@
         <v>0</v>
       </c>
       <c r="AB12" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:28" customHeight="1" ht="26">
       <c r="A13" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E13" s="8">
         <v>20.55015</v>
@@ -2564,10 +2549,10 @@
         <v>105.91104</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I13" s="9">
         <v>52000.0</v>
@@ -2579,7 +2564,7 @@
         <v>9</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="M13" s="9">
         <v>600</v>
@@ -2594,7 +2579,7 @@
         <v>93.0</v>
       </c>
       <c r="Q13" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="R13" s="9">
         <v>72</v>
@@ -2627,12 +2612,12 @@
         <v>0</v>
       </c>
       <c r="AB13" s="7" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:28" customHeight="1" ht="26">
       <c r="A14" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>31</v>
@@ -2641,19 +2626,19 @@
         <v>48</v>
       </c>
       <c r="D14" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E14" s="8">
+        <v>20.444673</v>
+      </c>
+      <c r="F14" s="8">
+        <v>106.17272</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="H14" s="7" t="s">
         <v>111</v>
-      </c>
-      <c r="E14" s="8">
-        <v>20.429915</v>
-      </c>
-      <c r="F14" s="8">
-        <v>106.202506</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>113</v>
       </c>
       <c r="I14" s="9">
         <v>62000.0</v>
@@ -2665,7 +2650,7 @@
         <v>14</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="M14" s="9">
         <v>900</v>
@@ -2680,7 +2665,7 @@
         <v>96.5</v>
       </c>
       <c r="Q14" s="7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="R14" s="9">
         <v>102</v>
@@ -2713,21 +2698,21 @@
         <v>0</v>
       </c>
       <c r="AB14" s="7" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" spans="1:28" customHeight="1" ht="26">
       <c r="A15" s="7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B15" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E15" s="8">
         <v>20.607146</v>
@@ -2736,10 +2721,10 @@
         <v>105.932884</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I15" s="9">
         <v>40000.0</v>
@@ -2751,7 +2736,7 @@
         <v>10</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="M15" s="9">
         <v>1200</v>
@@ -2766,7 +2751,7 @@
         <v>98.0</v>
       </c>
       <c r="Q15" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="R15" s="9">
         <v>88</v>
@@ -2799,21 +2784,21 @@
         <v>0</v>
       </c>
       <c r="AB15" s="7" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" spans="1:28" customHeight="1" ht="26">
       <c r="A16" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E16" s="8">
         <v>20.4356</v>
@@ -2822,10 +2807,10 @@
         <v>106.1754</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I16" s="9">
         <v>48000.0</v>
@@ -2837,7 +2822,7 @@
         <v>12</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="M16" s="9">
         <v>500</v>
@@ -2852,7 +2837,7 @@
         <v>94.0</v>
       </c>
       <c r="Q16" s="7" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="R16" s="9">
         <v>68</v>
@@ -2885,12 +2870,12 @@
         <v>0</v>
       </c>
       <c r="AB16" s="7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:28" customHeight="1" ht="26">
       <c r="A17" s="7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B17" s="8" t="s">
         <v>31</v>
@@ -2899,7 +2884,7 @@
         <v>48</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E17" s="8">
         <v>20.4312</v>
@@ -2908,10 +2893,10 @@
         <v>106.1824</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I17" s="9">
         <v>50000.0</v>
@@ -2923,7 +2908,7 @@
         <v>6</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="M17" s="9">
         <v>550</v>
@@ -2938,7 +2923,7 @@
         <v>92.0</v>
       </c>
       <c r="Q17" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="R17" s="9">
         <v>82</v>
@@ -2971,33 +2956,33 @@
         <v>0</v>
       </c>
       <c r="AB17" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:28" customHeight="1" ht="26">
       <c r="A18" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="E18" s="8">
+        <v>20.37461</v>
+      </c>
+      <c r="F18" s="8">
+        <v>106.134744</v>
+      </c>
+      <c r="G18" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D18" s="7" t="s">
+      <c r="H18" s="7" t="s">
         <v>140</v>
-      </c>
-      <c r="E18" s="8">
-        <v>20.409575</v>
-      </c>
-      <c r="F18" s="8">
-        <v>106.14908200000001</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>142</v>
       </c>
       <c r="I18" s="9">
         <v>32000.0</v>
@@ -3009,7 +2994,7 @@
         <v>6</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="M18" s="9">
         <v>400</v>
@@ -3024,7 +3009,7 @@
         <v>93.0</v>
       </c>
       <c r="Q18" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="R18" s="9">
         <v>45</v>
@@ -3057,33 +3042,33 @@
         <v>0</v>
       </c>
       <c r="AB18" s="7" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" spans="1:28" customHeight="1" ht="26">
       <c r="A19" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="B19" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="C19" s="7" t="s">
+      <c r="E19" s="8">
+        <v>20.405</v>
+      </c>
+      <c r="F19" s="8">
+        <v>106.215</v>
+      </c>
+      <c r="G19" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="H19" s="7" t="s">
         <v>148</v>
-      </c>
-      <c r="E19" s="8">
-        <v>20.396133</v>
-      </c>
-      <c r="F19" s="8">
-        <v>106.213331</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>150</v>
       </c>
       <c r="I19" s="9">
         <v>28000.0</v>
@@ -3095,7 +3080,7 @@
         <v>5</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="M19" s="9">
         <v>350</v>
@@ -3110,7 +3095,7 @@
         <v>91.5</v>
       </c>
       <c r="Q19" s="7" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="R19" s="9">
         <v>38</v>
@@ -3143,33 +3128,33 @@
         <v>0</v>
       </c>
       <c r="AB19" s="7" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="20" spans="1:28" customHeight="1" ht="26">
       <c r="A20" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="E20" s="8">
+        <v>20.26515</v>
+      </c>
+      <c r="F20" s="8">
+        <v>105.942854</v>
+      </c>
+      <c r="G20" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="C20" s="7" t="s">
+      <c r="H20" s="7" t="s">
         <v>155</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="E20" s="8">
-        <v>20.249714</v>
-      </c>
-      <c r="F20" s="8">
-        <v>105.995138</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>158</v>
       </c>
       <c r="I20" s="9">
         <v>30000.0</v>
@@ -3181,7 +3166,7 @@
         <v>7</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="M20" s="9">
         <v>420</v>
@@ -3196,7 +3181,7 @@
         <v>94.5</v>
       </c>
       <c r="Q20" s="7" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="R20" s="9">
         <v>48</v>
@@ -3229,21 +3214,21 @@
         <v>0</v>
       </c>
       <c r="AB20" s="7" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:28" customHeight="1" ht="26">
       <c r="A21" s="7" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E21" s="8">
         <v>20.458024</v>
@@ -3252,10 +3237,10 @@
         <v>106.187597</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="I21" s="9">
         <v>22000.0</v>
@@ -3267,7 +3252,7 @@
         <v>4</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="M21" s="9">
         <v>280</v>
@@ -3282,7 +3267,7 @@
         <v>90.0</v>
       </c>
       <c r="Q21" s="7" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="R21" s="9">
         <v>32</v>
@@ -3315,21 +3300,21 @@
         <v>0</v>
       </c>
       <c r="AB21" s="7" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="22" spans="1:28" customHeight="1" ht="26">
       <c r="A22" s="7" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>48</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E22" s="8">
         <v>20.4421</v>
@@ -3338,10 +3323,10 @@
         <v>106.1765</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="I22" s="9">
         <v>26000.0</v>
@@ -3353,7 +3338,7 @@
         <v>6</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="M22" s="9">
         <v>380</v>
@@ -3368,7 +3353,7 @@
         <v>93.5</v>
       </c>
       <c r="Q22" s="7" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="R22" s="9">
         <v>42</v>
@@ -3401,21 +3386,21 @@
         <v>0</v>
       </c>
       <c r="AB22" s="7" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="23" spans="1:28" customHeight="1" ht="26">
       <c r="A23" s="7" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E23" s="8">
         <v>20.36133</v>
@@ -3424,10 +3409,10 @@
         <v>105.909392</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="I23" s="9">
         <v>34000.0</v>
@@ -3439,7 +3424,7 @@
         <v>7</v>
       </c>
       <c r="L23" s="7" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="M23" s="9">
         <v>420</v>
@@ -3454,7 +3439,7 @@
         <v>95.0</v>
       </c>
       <c r="Q23" s="7" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="R23" s="9">
         <v>46</v>
@@ -3487,21 +3472,21 @@
         <v>0</v>
       </c>
       <c r="AB23" s="7" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="24" spans="1:28" customHeight="1" ht="26">
       <c r="A24" s="7" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E24" s="8">
         <v>20.3556</v>
@@ -3510,10 +3495,10 @@
         <v>105.91240000000001</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="I24" s="9">
         <v>28000.0</v>
@@ -3525,7 +3510,7 @@
         <v>5</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="M24" s="9">
         <v>300</v>
@@ -3540,7 +3525,7 @@
         <v>91.0</v>
       </c>
       <c r="Q24" s="7" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="R24" s="9">
         <v>34</v>
@@ -3573,21 +3558,21 @@
         <v>0</v>
       </c>
       <c r="AB24" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="25" spans="1:28" customHeight="1" ht="26">
       <c r="A25" s="7" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>193</v>
+        <v>94</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="E25" s="8">
         <v>20.5215</v>
@@ -3596,10 +3581,10 @@
         <v>105.9284</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="I25" s="9">
         <v>25000.0</v>
@@ -3611,7 +3596,7 @@
         <v>5</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="M25" s="9">
         <v>360</v>
@@ -3626,7 +3611,7 @@
         <v>94.0</v>
       </c>
       <c r="Q25" s="7" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="R25" s="9">
         <v>40</v>
@@ -3659,21 +3644,21 @@
         <v>0</v>
       </c>
       <c r="AB25" s="7" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="26" spans="1:28" customHeight="1" ht="26">
       <c r="A26" s="7" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>201</v>
+        <v>175</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="E26" s="8">
         <v>20.3421</v>
@@ -3682,10 +3667,10 @@
         <v>105.9234</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="I26" s="9">
         <v>30000.0</v>
@@ -3697,7 +3682,7 @@
         <v>6</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="M26" s="9">
         <v>320</v>
@@ -3712,7 +3697,7 @@
         <v>92.5</v>
       </c>
       <c r="Q26" s="7" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="R26" s="9">
         <v>36</v>
@@ -3745,7 +3730,7 @@
         <v>0</v>
       </c>
       <c r="AB26" s="7" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -3782,326 +3767,326 @@
   <sheetData>
     <row r="1" spans="1:3" customHeight="1" ht="30">
       <c r="A1" s="10" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3" spans="1:3" customHeight="1" ht="28">
       <c r="A3" s="1" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:3" customHeight="1" ht="24">
       <c r="A4" s="11" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:3" customHeight="1" ht="24">
       <c r="A5" s="11" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:3" customHeight="1" ht="24">
       <c r="A6" s="11" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" spans="1:3" customHeight="1" ht="24">
       <c r="A7" s="11" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" spans="1:3" customHeight="1" ht="24">
       <c r="A8" s="11" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" spans="1:3" customHeight="1" ht="24">
       <c r="A9" s="11" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10" spans="1:3" customHeight="1" ht="24">
       <c r="A10" s="11" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
     </row>
     <row r="11" spans="1:3" customHeight="1" ht="24">
       <c r="A11" s="11" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12" spans="1:3" customHeight="1" ht="24">
       <c r="A12" s="11" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:3" customHeight="1" ht="24">
       <c r="A13" s="11" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
     </row>
     <row r="14" spans="1:3" customHeight="1" ht="24">
       <c r="A14" s="11" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="15" spans="1:3" customHeight="1" ht="24">
       <c r="A15" s="11" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
     </row>
     <row r="16" spans="1:3" customHeight="1" ht="24">
       <c r="A16" s="11" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
     </row>
     <row r="17" spans="1:3" customHeight="1" ht="24">
       <c r="A17" s="11" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="18" spans="1:3" customHeight="1" ht="24">
       <c r="A18" s="11" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
     </row>
     <row r="19" spans="1:3" customHeight="1" ht="24">
       <c r="A19" s="11" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
     </row>
     <row r="20" spans="1:3" customHeight="1" ht="24">
       <c r="A20" s="11" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
     </row>
     <row r="21" spans="1:3" customHeight="1" ht="24">
       <c r="A21" s="11" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="22" spans="1:3" customHeight="1" ht="24">
       <c r="A22" s="11" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
     </row>
     <row r="23" spans="1:3" customHeight="1" ht="24">
       <c r="A23" s="11" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="24" spans="1:3" customHeight="1" ht="24">
       <c r="A24" s="11" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
     </row>
     <row r="25" spans="1:3" customHeight="1" ht="24">
       <c r="A25" s="11" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
     </row>
     <row r="26" spans="1:3" customHeight="1" ht="24">
       <c r="A26" s="11" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
     </row>
     <row r="27" spans="1:3" customHeight="1" ht="24">
       <c r="A27" s="11" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="28" spans="1:3" customHeight="1" ht="24">
       <c r="A28" s="11" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="29" spans="1:3" customHeight="1" ht="24">
       <c r="A29" s="11" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
     </row>
     <row r="30" spans="1:3" customHeight="1" ht="24">
       <c r="A30" s="11" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
     </row>
     <row r="31" spans="1:3" customHeight="1" ht="24">
       <c r="A31" s="11" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -4128,18 +4113,18 @@
   <sheetData>
     <row r="1" spans="1:2" customHeight="1" ht="28">
       <c r="A1" s="1" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:2" customHeight="1" ht="22">
       <c r="A2" s="2" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:2" customHeight="1" ht="22">
@@ -4147,86 +4132,86 @@
         <v>31</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
     </row>
     <row r="4" spans="1:2" customHeight="1" ht="22">
       <c r="A4" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
     </row>
     <row r="5" spans="1:2" customHeight="1" ht="22">
       <c r="A5" s="2" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:2" customHeight="1" ht="22">
       <c r="A6" s="2" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7" spans="1:2" customHeight="1" ht="22">
       <c r="B7" s="2" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="8" spans="1:2" customHeight="1" ht="22">
       <c r="B8" s="2" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
     </row>
     <row r="9" spans="1:2" customHeight="1" ht="22">
       <c r="B9" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:2" customHeight="1" ht="22">
       <c r="B10" s="2" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:2" customHeight="1" ht="22">
       <c r="B11" s="2" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:2" customHeight="1" ht="22">
       <c r="B12" s="2" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13" spans="1:2" customHeight="1" ht="22">
       <c r="B13" s="2" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
     </row>
     <row r="14" spans="1:2" customHeight="1" ht="22">
       <c r="B14" s="2" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" spans="1:2" customHeight="1" ht="22">
       <c r="B15" s="2" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="16" spans="1:2" customHeight="1" ht="22">
       <c r="B16" s="2" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="17" spans="1:2" customHeight="1" ht="22">
       <c r="B17" s="2" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="18" spans="1:2" customHeight="1" ht="22">
@@ -4236,37 +4221,37 @@
     </row>
     <row r="19" spans="1:2" customHeight="1" ht="22">
       <c r="B19" s="2" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
     </row>
     <row r="20" spans="1:2" customHeight="1" ht="22">
       <c r="B20" s="2" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
     </row>
     <row r="21" spans="1:2" customHeight="1" ht="22">
       <c r="B21" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:2" customHeight="1" ht="22">
       <c r="B22" s="2" t="s">
-        <v>103</v>
+        <v>283</v>
       </c>
     </row>
     <row r="23" spans="1:2" customHeight="1" ht="22">
       <c r="B23" s="2" t="s">
-        <v>288</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:2" customHeight="1" ht="22">
       <c r="B24" s="2" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
     </row>
     <row r="25" spans="1:2" customHeight="1" ht="22">
       <c r="B25" s="2" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
     </row>
     <row r="26" spans="1:2" customHeight="1" ht="22">
@@ -4276,522 +4261,522 @@
     </row>
     <row r="27" spans="1:2" customHeight="1" ht="22">
       <c r="B27" s="2" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="28" spans="1:2" customHeight="1" ht="22">
       <c r="B28" s="2" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
     </row>
     <row r="29" spans="1:2" customHeight="1" ht="22">
       <c r="B29" s="2" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
     </row>
     <row r="30" spans="1:2" customHeight="1" ht="22">
       <c r="B30" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31" spans="1:2" customHeight="1" ht="22">
       <c r="B31" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="32" spans="1:2" customHeight="1" ht="22">
       <c r="B32" s="2" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
     </row>
     <row r="33" spans="1:2" customHeight="1" ht="22">
       <c r="B33" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="34" spans="1:2" customHeight="1" ht="22">
       <c r="B34" s="2" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
     </row>
     <row r="35" spans="1:2" customHeight="1" ht="22">
       <c r="B35" s="2" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
     </row>
     <row r="36" spans="1:2" customHeight="1" ht="22">
       <c r="B36" s="2" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
     </row>
     <row r="37" spans="1:2" customHeight="1" ht="22">
       <c r="B37" s="2" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
     </row>
     <row r="38" spans="1:2" customHeight="1" ht="22">
       <c r="B38" s="2" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
     </row>
     <row r="39" spans="1:2" customHeight="1" ht="22">
       <c r="B39" s="2" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
     </row>
     <row r="40" spans="1:2" customHeight="1" ht="22">
       <c r="B40" s="2" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
     </row>
     <row r="41" spans="1:2" customHeight="1" ht="22">
       <c r="B41" s="2" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
     </row>
     <row r="42" spans="1:2" customHeight="1" ht="22">
       <c r="B42" s="2" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
     </row>
     <row r="43" spans="1:2" customHeight="1" ht="22">
       <c r="B43" s="2" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
     </row>
     <row r="44" spans="1:2" customHeight="1" ht="22">
       <c r="B44" s="2" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="45" spans="1:2" customHeight="1" ht="22">
       <c r="B45" s="2" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
     </row>
     <row r="46" spans="1:2" customHeight="1" ht="22">
       <c r="B46" s="2" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
     </row>
     <row r="47" spans="1:2" customHeight="1" ht="22">
       <c r="B47" s="2" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
     </row>
     <row r="48" spans="1:2" customHeight="1" ht="22">
       <c r="B48" s="2" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
     </row>
     <row r="49" spans="1:2" customHeight="1" ht="22">
       <c r="B49" s="2" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
     </row>
     <row r="50" spans="1:2" customHeight="1" ht="22">
       <c r="B50" s="2" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
     </row>
     <row r="51" spans="1:2" customHeight="1" ht="22">
       <c r="B51" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
     </row>
     <row r="52" spans="1:2" customHeight="1" ht="22">
       <c r="B52" s="2" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="53" spans="1:2" customHeight="1" ht="22">
       <c r="B53" s="2" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
     </row>
     <row r="54" spans="1:2" customHeight="1" ht="22">
       <c r="B54" s="2" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
     </row>
     <row r="55" spans="1:2" customHeight="1" ht="22">
       <c r="B55" s="2" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
     </row>
     <row r="56" spans="1:2" customHeight="1" ht="22">
       <c r="B56" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
     </row>
     <row r="57" spans="1:2" customHeight="1" ht="22">
       <c r="B57" s="2" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
     </row>
     <row r="58" spans="1:2" customHeight="1" ht="22">
       <c r="B58" s="2" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
     </row>
     <row r="59" spans="1:2" customHeight="1" ht="22">
       <c r="B59" s="2" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
     </row>
     <row r="60" spans="1:2" customHeight="1" ht="22">
       <c r="B60" s="2" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
     </row>
     <row r="61" spans="1:2" customHeight="1" ht="22">
       <c r="B61" s="2" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
     </row>
     <row r="62" spans="1:2" customHeight="1" ht="22">
       <c r="B62" s="2" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="63" spans="1:2" customHeight="1" ht="22">
       <c r="B63" s="2" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
     </row>
     <row r="64" spans="1:2" customHeight="1" ht="22">
       <c r="B64" s="2" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
     </row>
     <row r="65" spans="1:2" customHeight="1" ht="22">
       <c r="B65" s="2" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="66" spans="1:2" customHeight="1" ht="22">
       <c r="B66" s="2" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
     </row>
     <row r="67" spans="1:2" customHeight="1" ht="22">
       <c r="B67" s="2" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
     </row>
     <row r="68" spans="1:2" customHeight="1" ht="22">
       <c r="B68" s="2" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
     </row>
     <row r="69" spans="1:2" customHeight="1" ht="22">
       <c r="B69" s="2" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
     </row>
     <row r="70" spans="1:2" customHeight="1" ht="22">
       <c r="B70" s="2" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
     </row>
     <row r="71" spans="1:2" customHeight="1" ht="22">
       <c r="B71" s="2" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
     </row>
     <row r="72" spans="1:2" customHeight="1" ht="22">
       <c r="B72" s="2" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
     </row>
     <row r="73" spans="1:2" customHeight="1" ht="22">
       <c r="B73" s="2" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
     </row>
     <row r="74" spans="1:2" customHeight="1" ht="22">
       <c r="B74" s="2" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
     </row>
     <row r="75" spans="1:2" customHeight="1" ht="22">
       <c r="B75" s="2" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
     </row>
     <row r="76" spans="1:2" customHeight="1" ht="22">
       <c r="B76" s="2" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="77" spans="1:2" customHeight="1" ht="22">
       <c r="B77" s="2" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
     </row>
     <row r="78" spans="1:2" customHeight="1" ht="22">
       <c r="B78" s="2" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
     </row>
     <row r="79" spans="1:2" customHeight="1" ht="22">
       <c r="B79" s="2" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
     </row>
     <row r="80" spans="1:2" customHeight="1" ht="22">
       <c r="B80" s="2" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="81" spans="1:2" customHeight="1" ht="22">
       <c r="B81" s="2" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
     </row>
     <row r="82" spans="1:2" customHeight="1" ht="22">
       <c r="B82" s="2" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
     </row>
     <row r="83" spans="1:2" customHeight="1" ht="22">
       <c r="B83" s="2" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
     </row>
     <row r="84" spans="1:2" customHeight="1" ht="22">
       <c r="B84" s="2" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
     </row>
     <row r="85" spans="1:2" customHeight="1" ht="22">
       <c r="B85" s="2" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
     </row>
     <row r="86" spans="1:2" customHeight="1" ht="22">
       <c r="B86" s="2" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
     </row>
     <row r="87" spans="1:2" customHeight="1" ht="22">
       <c r="B87" s="2" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
     </row>
     <row r="88" spans="1:2" customHeight="1" ht="22">
       <c r="B88" s="2" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
     </row>
     <row r="89" spans="1:2" customHeight="1" ht="22">
       <c r="B89" s="2" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
     </row>
     <row r="90" spans="1:2" customHeight="1" ht="22">
       <c r="B90" s="2" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
     </row>
     <row r="91" spans="1:2" customHeight="1" ht="22">
       <c r="B91" s="2" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
     </row>
     <row r="92" spans="1:2" customHeight="1" ht="22">
       <c r="B92" s="2" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
     </row>
     <row r="93" spans="1:2" customHeight="1" ht="22">
       <c r="B93" s="2" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="94" spans="1:2" customHeight="1" ht="22">
       <c r="B94" s="2" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
     </row>
     <row r="95" spans="1:2" customHeight="1" ht="22">
       <c r="B95" s="2" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
     </row>
     <row r="96" spans="1:2" customHeight="1" ht="22">
       <c r="B96" s="2" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
     </row>
     <row r="97" spans="1:2" customHeight="1" ht="22">
       <c r="B97" s="2" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
     </row>
     <row r="98" spans="1:2" customHeight="1" ht="22">
       <c r="B98" s="2" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
     </row>
     <row r="99" spans="1:2" customHeight="1" ht="22">
       <c r="B99" s="2" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
     </row>
     <row r="100" spans="1:2" customHeight="1" ht="22">
       <c r="B100" s="2" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
     </row>
     <row r="101" spans="1:2" customHeight="1" ht="22">
       <c r="B101" s="2" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="102" spans="1:2" customHeight="1" ht="22">
       <c r="B102" s="2" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
     </row>
     <row r="103" spans="1:2" customHeight="1" ht="22">
       <c r="B103" s="2" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
     </row>
     <row r="104" spans="1:2" customHeight="1" ht="22">
       <c r="B104" s="2" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
     </row>
     <row r="105" spans="1:2" customHeight="1" ht="22">
       <c r="B105" s="2" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
     </row>
     <row r="106" spans="1:2" customHeight="1" ht="22">
       <c r="B106" s="2" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
     </row>
     <row r="107" spans="1:2" customHeight="1" ht="22">
       <c r="B107" s="2" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
     </row>
     <row r="108" spans="1:2" customHeight="1" ht="22">
       <c r="B108" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
     </row>
     <row r="109" spans="1:2" customHeight="1" ht="22">
       <c r="B109" s="2" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
     </row>
     <row r="110" spans="1:2" customHeight="1" ht="22">
       <c r="B110" s="2" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
     </row>
     <row r="111" spans="1:2" customHeight="1" ht="22">
       <c r="B111" s="2" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
     </row>
     <row r="112" spans="1:2" customHeight="1" ht="22">
       <c r="B112" s="2" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
     </row>
     <row r="113" spans="1:2" customHeight="1" ht="22">
       <c r="B113" s="2" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
     </row>
     <row r="114" spans="1:2" customHeight="1" ht="22">
       <c r="B114" s="2" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
     </row>
     <row r="115" spans="1:2" customHeight="1" ht="22">
       <c r="B115" s="2" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
     </row>
     <row r="116" spans="1:2" customHeight="1" ht="22">
       <c r="B116" s="2" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
     </row>
     <row r="117" spans="1:2" customHeight="1" ht="22">
       <c r="B117" s="2" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
     </row>
     <row r="118" spans="1:2" customHeight="1" ht="22">
       <c r="B118" s="2" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
     </row>
     <row r="119" spans="1:2" customHeight="1" ht="22">
       <c r="B119" s="2" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
     </row>
     <row r="120" spans="1:2" customHeight="1" ht="22">
       <c r="B120" s="2" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
     </row>
     <row r="121" spans="1:2" customHeight="1" ht="22">
       <c r="B121" s="2" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
     </row>
     <row r="122" spans="1:2" customHeight="1" ht="22">
       <c r="B122" s="2" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
     </row>
     <row r="123" spans="1:2" customHeight="1" ht="22">
       <c r="B123" s="2" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
     </row>
     <row r="124" spans="1:2" customHeight="1" ht="22">
       <c r="B124" s="2" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
     </row>
     <row r="125" spans="1:2" customHeight="1" ht="22">
       <c r="B125" s="2" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
     </row>
     <row r="126" spans="1:2" customHeight="1" ht="22">
       <c r="B126" s="2" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
     </row>
     <row r="127" spans="1:2" customHeight="1" ht="22">
       <c r="B127" s="2" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
     </row>
     <row r="128" spans="1:2" customHeight="1" ht="22">
       <c r="B128" s="2" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
     </row>
     <row r="129" spans="1:2" customHeight="1" ht="22">
       <c r="B129" s="2" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="130" spans="1:2" customHeight="1" ht="22">
       <c r="B130" s="2" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
     </row>
   </sheetData>

</xml_diff>